<commit_message>
add more information to file MENU
</commit_message>
<xml_diff>
--- a/public/menu.xlsx
+++ b/public/menu.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FrontEnd\healthy_eating\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1E6E23-041A-4F61-A78D-D6F42C4EC088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13FB1A4A-784E-4AA6-8179-2F5B9C5BAEAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,16 +25,277 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t>TEST MENU</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="88">
+  <si>
+    <t>Week / Section</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Meal</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Gourmet</t>
+  </si>
+  <si>
+    <t>Alfredo Penne with Broccoli</t>
+  </si>
+  <si>
+    <t>Baked Chicken</t>
+  </si>
+  <si>
+    <t>Chicken &amp; Mushroom Marsala</t>
+  </si>
+  <si>
+    <t>Chicken Pot Pie</t>
+  </si>
+  <si>
+    <t>Country Fried Chicken &amp; Gravy</t>
+  </si>
+  <si>
+    <t>Fettuccini Alfredo</t>
+  </si>
+  <si>
+    <t>Sweet Sesame Chicken</t>
+  </si>
+  <si>
+    <t>Chicken with Brown Rice</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>Comfort</t>
+  </si>
+  <si>
+    <t>Romano Crusted Chicken</t>
+  </si>
+  <si>
+    <t>Grilled Chicken Marinara w/ Parmesan</t>
+  </si>
+  <si>
+    <t>Green Pepper Steak</t>
+  </si>
+  <si>
+    <t>Lasagna w/ Meat Sauce</t>
+  </si>
+  <si>
+    <t>Spaghetti w/ Meatballs</t>
+  </si>
+  <si>
+    <t>Fried Chicken</t>
+  </si>
+  <si>
+    <t>Lemongrass Basil Chicken</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>Deli</t>
+  </si>
+  <si>
+    <t>Adobo Chicken</t>
+  </si>
+  <si>
+    <t>Beef Teriyaki</t>
+  </si>
+  <si>
+    <t>Chicken Parmesan</t>
+  </si>
+  <si>
+    <t>General Tso's Chicken</t>
+  </si>
+  <si>
+    <t>Chicken Enchilada</t>
+  </si>
+  <si>
+    <t>Fresh Bread Cheese Pizza</t>
+  </si>
+  <si>
+    <t>Spinach, Rice &amp; Beans Enchilada</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>International</t>
+  </si>
+  <si>
+    <t>Pepper Jack Parmesan &amp; Mozzarella Cheese Stuffed Chicken</t>
+  </si>
+  <si>
+    <t>Fish Filet</t>
+  </si>
+  <si>
+    <t>Roast Turkey</t>
+  </si>
+  <si>
+    <t>French Bread Pepperoni Pizza</t>
+  </si>
+  <si>
+    <t>Grilled Chicken Sandwich</t>
+  </si>
+  <si>
+    <t>Uncured Pepperoni &amp; Cheese Chicken Nuggets</t>
+  </si>
+  <si>
+    <t>Salisbury Steak</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Family</t>
+  </si>
+  <si>
+    <t>Beef Merlot</t>
+  </si>
+  <si>
+    <t>Chicken Fettuccini Alfredo</t>
+  </si>
+  <si>
+    <t>Classic Mac &amp; Beef</t>
+  </si>
+  <si>
+    <t>Classic Meatloaf</t>
+  </si>
+  <si>
+    <t>Crustless Chicken Pot Pie</t>
+  </si>
+  <si>
+    <t>Tuna Noodle Casserole</t>
+  </si>
+  <si>
+    <t>Week 6</t>
+  </si>
+  <si>
+    <t>Homestyle</t>
+  </si>
+  <si>
+    <t>Beef Pot Pie</t>
+  </si>
+  <si>
+    <t>Chicken &amp; Broccoli Alfredo</t>
+  </si>
+  <si>
+    <t>Chicken à la King</t>
+  </si>
+  <si>
+    <t>Chicken Margherita w/ Balsamic</t>
+  </si>
+  <si>
+    <t>Creamed Chipped Beef</t>
+  </si>
+  <si>
+    <t>Glazed Turkey Tenderloins</t>
+  </si>
+  <si>
+    <t>Swedish Meatballs</t>
+  </si>
+  <si>
+    <t>Breakfast</t>
+  </si>
+  <si>
+    <t>Breakfast Burrito</t>
+  </si>
+  <si>
+    <t>Buttermilk Pancakes</t>
+  </si>
+  <si>
+    <t>Bacon, Egg &amp; Cheese on a Biscuit</t>
+  </si>
+  <si>
+    <t>Meat Lovers Breakfast Bowl</t>
+  </si>
+  <si>
+    <t>Sausage, Egg &amp; Cheese Croissant</t>
+  </si>
+  <si>
+    <t>Bacon, Egg &amp; Cheddar Cheese Sandwich</t>
+  </si>
+  <si>
+    <t>Bacon Breakfast Bowl</t>
+  </si>
+  <si>
+    <t>Bacon Ciabatta Cheese Tray</t>
+  </si>
+  <si>
+    <t>Salads</t>
+  </si>
+  <si>
+    <t>Chicken Caesar</t>
+  </si>
+  <si>
+    <t>Santa Fe Style w/ Chicken</t>
+  </si>
+  <si>
+    <t>Turkey Bacon &amp; Cobb</t>
+  </si>
+  <si>
+    <t>Spinach Dijon</t>
+  </si>
+  <si>
+    <t>Cranberry Walnut</t>
+  </si>
+  <si>
+    <t>Asian Style w/ Chicken</t>
+  </si>
+  <si>
+    <t>Vegetarian</t>
+  </si>
+  <si>
+    <t>Cheese Ravioli Bowl</t>
+  </si>
+  <si>
+    <t>Chili Mac Bowl</t>
+  </si>
+  <si>
+    <t>Buffalo Cauliflower Mac &amp; Cheese Bowl</t>
+  </si>
+  <si>
+    <t>General Tso's Tofu</t>
+  </si>
+  <si>
+    <t>Pad Thai</t>
+  </si>
+  <si>
+    <t>Organic Veggie Burgers</t>
+  </si>
+  <si>
+    <t>Santa Fe-Style Rice &amp; Beans</t>
+  </si>
+  <si>
+    <t>Gluten-Free</t>
+  </si>
+  <si>
+    <t>Lasagna Bowl</t>
+  </si>
+  <si>
+    <t>Mongolian Inspired Beef Bowl</t>
+  </si>
+  <si>
+    <t>Cheese Bacon Wrapped Stuffed Chicken</t>
+  </si>
+  <si>
+    <t>Veggie Loaf</t>
+  </si>
+  <si>
+    <t>Chicken Burrito Bowl</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -42,16 +303,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF08752E"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -59,12 +331,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD7E8D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -345,13 +632,868 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" customWidth="1"/>
+    <col min="3" max="3" width="50.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.44140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="2"/>
+    </row>
+    <row r="25" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" s="2"/>
+    </row>
+    <row r="27" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" s="2"/>
+    </row>
+    <row r="28" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" s="2"/>
+    </row>
+    <row r="29" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D34" s="2"/>
+    </row>
+    <row r="35" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D35" s="2"/>
+    </row>
+    <row r="36" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D38" s="2"/>
+    </row>
+    <row r="39" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D44" s="2"/>
+    </row>
+    <row r="45" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D45" s="2"/>
+    </row>
+    <row r="46" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D46" s="2"/>
+    </row>
+    <row r="47" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D47" s="2"/>
+    </row>
+    <row r="48" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D48" s="2"/>
+    </row>
+    <row r="49" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D49" s="2"/>
+    </row>
+    <row r="50" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D50" s="2"/>
+    </row>
+    <row r="51" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D51" s="2"/>
+    </row>
+    <row r="52" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D52" s="2"/>
+    </row>
+    <row r="53" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D53" s="2"/>
+    </row>
+    <row r="54" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D54" s="2"/>
+    </row>
+    <row r="55" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D55" s="2"/>
+    </row>
+    <row r="56" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D56" s="2"/>
+    </row>
+    <row r="57" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D57" s="2"/>
+    </row>
+    <row r="58" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D58" s="2"/>
+    </row>
+    <row r="59" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D59" s="2"/>
+    </row>
+    <row r="60" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D60" s="2"/>
+    </row>
+    <row r="61" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D61" s="2"/>
+    </row>
+    <row r="62" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D62" s="2"/>
+    </row>
+    <row r="63" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D63" s="2"/>
+    </row>
+    <row r="64" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D64" s="2"/>
+    </row>
+    <row r="65" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D65" s="2"/>
+    </row>
+    <row r="66" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D66" s="2"/>
+    </row>
+    <row r="67" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D67" s="2"/>
+    </row>
+    <row r="68" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D68" s="2"/>
+    </row>
+    <row r="69" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D69" s="2"/>
+    </row>
+    <row r="70" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D70" s="2"/>
+    </row>
+    <row r="71" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D71" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>